<commit_message>
[claude-session] TUI pre-launch commit
Session-Id: 1779696004-43854-4c6d2e7bc8ee
</commit_message>
<xml_diff>
--- a/conversational-search-cost-calculator.xlsx
+++ b/conversational-search-cost-calculator.xlsx
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -139,6 +139,7 @@
     <xf numFmtId="165" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -219,6 +220,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Calc v2</author>
+    <author>Calculator</author>
   </authors>
   <commentList>
     <comment ref="B4" authorId="0" shapeId="0">
@@ -285,18 +287,21 @@
 Fraction of searches where user actually clicks through and triggers T1.</t>
       </text>
     </comment>
-    <comment ref="B17" authorId="0" shapeId="0">
+    <comment ref="B17" authorId="1" shapeId="0">
       <text>
-        <t>Whether Bedrock prompt caching is used for the M7 composition payload.
-When No, all cache rows zero out.
-Only available for Sonnet 4.6 — must be No for GLM models.</t>
+        <t>Our Postgres-backed Turn-1 short-circuit cache.
+On HIT, the proxy skips the entire LangGraph dispatch.
+Works for ANY baseline model (Sonnet AND GLM).
+Default: Yes.
+Toggle No to model cost without M7 cache.</t>
       </text>
     </comment>
-    <comment ref="B18" authorId="0" shapeId="0">
+    <comment ref="B18" authorId="1" shapeId="0">
       <text>
-        <t>Fraction of Turn 1 calls that hit a warm cache entry.
+        <t>Fraction of Turn 1 calls that hit a warm M7 cache entry.
 Presets: LOW=20%, MID=50% (default), HIGH=70%.
-PLACEHOLDER — refine from production-traffic measurement.</t>
+PLACEHOLDER — refine from production-traffic measurement.
+Applies to ALL baseline models when M7 cache is enabled.</t>
       </text>
     </comment>
     <comment ref="B19" authorId="0" shapeId="0">
@@ -320,6 +325,14 @@
 GLM 4.7 = $0.60/$2.20 per 1M tokens in/out, NO Bedrock prompt caching.
 GLM 4.7 Flash = $0.07/$0.40 per 1M tokens in/out, NO Bedrock prompt caching.
 IMPORTANT: GLM region availability NOT modeled — verify procurement separately.</t>
+      </text>
+    </comment>
+    <comment ref="B22" authorId="1" shapeId="0">
+      <text>
+        <t>Provider-side prefix cache. 1.25x write / 0.1x read on cached portion.
+Sonnet 4.6 only — not available for GLM 4.7 or GLM 4.7 Flash.
+This is AUTOMATIC — there is nothing to toggle.
+Affects rows B55, B56 (cache write/read costs) and B67 (T2+T3 cache reads).</t>
       </text>
     </comment>
   </commentList>
@@ -834,7 +847,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>M7 cache enabled</t>
+          <t>Application cache (M7) enabled</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -851,7 +864,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>M7 cache hit rate (%)</t>
+          <t>Application cache (M7) hit rate (%)</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
@@ -912,6 +925,17 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>AWS Bedrock prompt caching (auto)</t>
+        </is>
+      </c>
+      <c r="B22" s="8">
+        <f>IF(B21="Sonnet 4.6","Active (provider supports)","Inactive (provider unsupported)")</f>
+        <v/>
+      </c>
+    </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
@@ -1230,16 +1254,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cache applies flag (cache=Yes AND Sonnet 4.6 AND eager)</t>
+          <t>Bedrock prefix cache applies flag (Sonnet 4.6 only)</t>
         </is>
       </c>
       <c r="B46" s="13">
-        <f>IF(AND(B17="Yes",B21="Sonnet 4.6",B15="eager"),1,0)</f>
+        <f>IF(B21="Sonnet 4.6",1,0)</f>
         <v/>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>1 = cache active; 0 = all cache rows zero (GLM or cache off or deferred)</t>
+          <t>1 = Sonnet selected → prefix cache active; 0 = GLM (no provider-side caching). Cache savings scale automatically with B51 firing multiplier.</t>
         </is>
       </c>
     </row>
@@ -1323,6 +1347,22 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>M7 application cache applies flag (M7=Yes)</t>
+        </is>
+      </c>
+      <c r="B52" s="27">
+        <f>IF(B17="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>1 = M7 toggle on → application cache active in any firing mode. Cache savings scale automatically with B51 firing multiplier.</t>
+        </is>
+      </c>
+    </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
@@ -1381,7 +1421,7 @@
         </is>
       </c>
       <c r="B57" s="14">
-        <f>B46*(B18/100)*(B60+B61)</f>
+        <f>B52*(B18/100)*(B60+B61)</f>
         <v/>
       </c>
       <c r="C57" t="inlineStr">
@@ -1397,12 +1437,12 @@
         </is>
       </c>
       <c r="B58" s="14">
-        <f>(B6-B28)*B10*B44/1000000*B51</f>
+        <f>IF(B46=1,(B6-B28)*B10*B44/1000000,B6*B10*B44/1000000)*B51</f>
         <v/>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>T1 dyn tokens/call x T1 calls x active input rate x firing multiplier</t>
+          <t>T1 input: for Sonnet (cache on) uses dynamic tokens (B6-B28); for GLM (no cache) charges full B6 tokens. Multiplied by firing mode.</t>
         </is>
       </c>
     </row>
@@ -1477,12 +1517,12 @@
         </is>
       </c>
       <c r="B63" s="14">
-        <f>B47*(B20/100)*B60</f>
+        <f>B47*(B20/100)*(B60+B61)</f>
         <v/>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>rejection_rate x T1 LLM subtotal — queries that never reach T1</t>
+          <t>Classifier rejection skips both LLM and guardrail evaluation. Savings = rejection_rate x (LLM cost + guardrail cost).</t>
         </is>
       </c>
     </row>
@@ -1536,12 +1576,12 @@
         </is>
       </c>
       <c r="B68" s="14">
-        <f>(B7-B28)*B11*B44/1000000</f>
+        <f>IF(B46=1,(B7-B28)*B11*B44/1000000,B7*B11*B44/1000000)</f>
         <v/>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>T2+T3 dyn tokens/call x T2+T3 calls x active input rate</t>
+          <t>T2+T3 input: for Sonnet uses dynamic tokens (B7-B28); for GLM (no cache) charges full B7 tokens. Engagement-rate-weighted at higher level.</t>
         </is>
       </c>
     </row>
@@ -1947,7 +1987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2259,158 +2299,172 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>GLM region availability not modeled</t>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Classifier net savings depend on cost basis</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>This calculator does NOT check whether GLM 4.7 is available in your deployment region. The operator must verify procurement separately before relying on GLM cost estimates.</t>
+          <t>The classifier saves money when rejection_rate x (T1 LLM cost + T1 guardrail cost) &gt; classifier_per_call_cost. With Sonnet baseline and 40% rejection, classifier saves ~$0.007/search vs its $0.00075 cost — clear net positive. With GLM 4.7 Flash (very cheap input), the LLM-cost savings alone don't cover the classifier; the model-agnostic guardrail savings are what tip it positive. If guardrails are disabled in your deployment, re-check whether classifier still nets save for cheap GLM models — formula in B62/B63.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>5-min cache TTL assumed hit</t>
+          <t>GLM region availability not modeled</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>If a conversation resumes after 5 minutes, the cache-write cost is charged again.</t>
+          <t>This calculator does NOT check whether GLM 4.7 is available in your deployment region. The operator must verify procurement separately before relying on GLM cost estimates.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>LLM calls per turn default</t>
+          <t>5-min cache TTL assumed hit</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Default 1.1 for T1 leaves headroom; benchmark median is ~1 for the happy path, ~2 on retry/long-form (10%). Adjust B10 to match measured production cadence.</t>
+          <t>If a conversation resumes after 5 minutes, the cache-write cost is charged again.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Chars per token = 4 approximate</t>
+          <t>LLM calls per turn default</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Used only for guardrail text-unit math (not LLM billing). JSON content has a lower ratio.</t>
+          <t>Default 1.1 for T1 leaves headroom; benchmark median is ~1 for the happy path, ~2 on retry/long-form (10%). Adjust B10 to match measured production cadence.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
+          <t>Chars per token = 4 approximate</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Used only for guardrail text-unit math (not LLM billing). JSON content has a lower ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
           <t>Verifier LLM call not modeled</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>verify_search_intent runs per turn as a separate Bedrock call (~670 tok input). Add ~$0.0001/turn if enabled and material.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
         <is>
           <t>Where to Look (guardrail precision)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Go to Amazon Bedrock -&gt; Guardrails in the production region.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2.</t>
+          <t>1.</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Find guardrail ID lxv6kzi6cryg.</t>
+          <t>Go to Amazon Bedrock -&gt; Guardrails in the production region.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>3.</t>
+          <t>2.</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Check which policy types are enabled: Content Filters, Sensitive Information (PII), Contextual Grounding Check.</t>
+          <t>Find guardrail ID lxv6kzi6cryg.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Check which policy types are enabled: Content Filters, Sensitive Information (PII), Contextual Grounding Check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>Update the Guardrail policy mix dropdown in the calculator accordingly.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="16" t="inlineStr">
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t>Pricing Sources</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>AWS Bedrock pricing</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>https://aws.amazon.com/bedrock/pricing/ (fetched 2026-05-14)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Anthropic prompt-caching docs</t>
+          <t>AWS Bedrock pricing</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://docs.anthropic.com/en/docs/build-with-claude/prompt-caching (fetched 2026-05-14)</t>
+          <t>https://aws.amazon.com/bedrock/pricing/ (fetched 2026-05-14)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
+          <t>Anthropic prompt-caching docs</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://docs.anthropic.com/en/docs/build-with-claude/prompt-caching (fetched 2026-05-14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
           <t>GLM 4.7 model card (AWS Bedrock)</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>https://docs.aws.amazon.com/bedrock/latest/userguide/model-card-zai-glm-4-7.html</t>
         </is>

</xml_diff>